<commit_message>
Update gh-pages to output generated at 456a3b4
</commit_message>
<xml_diff>
--- a/上海-漫展信息.xlsx
+++ b/上海-漫展信息.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,7 +501,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="G2" t="n">
         <v>9.9</v>
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1976</v>
+        <v>1979</v>
       </c>
       <c r="G5" t="n">
         <v>98</v>
@@ -646,38 +646,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-10-26</t>
+          <t>2024-10-18</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·Nova次元动漫嘉年华</t>
+          <t>上海·幻境尘影—无期迷途光影展</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>沪光东路118号 昌格科技园北(沪光东路北)</t>
+          <t>陆家嘴西路168号 上海正大广场</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.10.26 09:00-10.27 18:00</t>
+          <t>2024.10.18 00:00-11.30 23:59</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1343</v>
+        <v>1979</v>
       </c>
       <c r="G6" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92899</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93269</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/mVcr4uCt1728896455696.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/kq6Pmpkv1728728206204.png</t>
         </is>
       </c>
     </row>
@@ -692,33 +692,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·杜莎夫人蜡像馆万圣节奇妙周x次元动漫嘉年华</t>
+          <t>上海·Nova次元动漫嘉年华</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>南京西路新世界商厦10层 上海杜莎夫人蜡像馆</t>
+          <t>沪光东路118号 昌格科技园北(沪光东路北)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.10.26 16:00-11.01 21:00</t>
+          <t>2024.10.26 09:00-10.27 18:00</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>8</v>
+        <v>1346</v>
       </c>
       <c r="G7" t="n">
-        <v>99</v>
+        <v>89</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93728</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92899</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/DzsWUuCu1729479657498.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/mVcr4uCt1728896455696.jpeg</t>
         </is>
       </c>
     </row>
@@ -733,35 +733,33 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·第五人格同人only</t>
+          <t>上海·杜莎夫人蜡像馆万圣节奇妙周x次元动漫嘉年华</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>柳营路125号明凯大厦 上海灯具城</t>
+          <t>南京西路新世界商厦10层 上海杜莎夫人蜡像馆</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.10.26 10:00-10.26 17:00</t>
+          <t>2024.10.26 16:00-11.01 21:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1610</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>已售罄</t>
-        </is>
+        <v>8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>99</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92128</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93728</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/0HZsXHtf1728977161010.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/DzsWUuCu1729479657498.jpeg</t>
         </is>
       </c>
     </row>
@@ -776,35 +774,35 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·第五届哈利波特ONLY同人展</t>
+          <t>上海·第五人格同人only</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>杨高中路2112号 界龙总部园</t>
+          <t>柳营路125号明凯大厦 上海灯具城</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.10.26 11:00-10.27 18:00</t>
+          <t>2024.10.26 10:00-10.26 17:00</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>37</v>
+        <v>1611</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>不可售</t>
+          <t>已售罄</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93090</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92128</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/fpCky5lW1727676129487.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/0HZsXHtf1728977161010.jpeg</t>
         </is>
       </c>
     </row>
@@ -819,21 +817,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·首届iPR动漫游戏嘉年华（取消）</t>
+          <t>上海·第五届哈利波特ONLY同人展</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>杨高中路2112号 界龙总部园</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.10.26 11:00-10.27 16:00</t>
+          <t>2024.10.26 11:00-10.27 18:00</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>883</v>
+        <v>37</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -842,12 +840,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=90989</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93090</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/5a8j0q361728699256113.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/fpCky5lW1727676129487.png</t>
         </is>
       </c>
     </row>
@@ -857,38 +855,40 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-10-27</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·“VWonderland万圣派对”虚拟主播见面会</t>
+          <t>上海·首届iPR动漫游戏嘉年华（取消）</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>苏虹路266号 魔法魅影•沉浸式Live剧场</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.10.27 10:00-10.27 22:00</t>
+          <t>2024.10.26 11:00-10.27 16:00</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>30</v>
-      </c>
-      <c r="G11" t="n">
-        <v>30</v>
+        <v>883</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93298</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=90989</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/Dh8Mytgq1728637643173.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/5a8j0q361728699256113.jpeg</t>
         </is>
       </c>
     </row>
@@ -898,38 +898,38 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2024-10-31</t>
+          <t>2024-10-27</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海 ·《天官赐福》动画四周年纪念展</t>
+          <t>上海·“VWonderland万圣派对”虚拟主播见面会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>南京西路2-68号 上海新世界城</t>
+          <t>苏虹路266号 魔法魅影•沉浸式Live剧场</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.10.31 00:00-11.30 23:59</t>
+          <t>2024.10.27 10:00-10.27 22:00</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1860</v>
+        <v>31</v>
       </c>
       <c r="G12" t="n">
-        <v>9.9</v>
+        <v>30</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92995</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93298</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/BJWdBkrc1727422599776.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/Dh8Mytgq1728637643173.png</t>
         </is>
       </c>
     </row>
@@ -944,33 +944,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·JinkyHuang x Hello Kitty 「柘柘之境」</t>
+          <t>上海 ·《天官赐福》动画四周年纪念展</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>淮海中路523号TX淮海F2层 BIP.Gallery</t>
+          <t>南京西路2-68号 上海新世界城</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.10.31 11:00-2025.02.28 21:00</t>
+          <t>2024.10.31 00:00-11.30 23:59</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>5</v>
+        <v>1866</v>
       </c>
       <c r="G13" t="n">
-        <v>68</v>
+        <v>9.9</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93594</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92995</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/uIC27Eyw1729150170638.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/BJWdBkrc1727422599776.jpeg</t>
         </is>
       </c>
     </row>
@@ -980,38 +980,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>2024-10-31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·JOing动漫游戏嘉年华</t>
+          <t>上海·JinkyHuang x Hello Kitty 「柘柘之境」</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>申虹路663号 虹桥协信中心</t>
+          <t>淮海中路523号TX淮海F2层 BIP.Gallery</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.11.02 10:00-11.03 17:00</t>
+          <t>2024.10.31 11:00-2025.02.28 21:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1884</v>
+        <v>6</v>
       </c>
       <c r="G14" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93044</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93594</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/GwoLrudT1728526473661.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/uIC27Eyw1729150170638.jpeg</t>
         </is>
       </c>
     </row>
@@ -1026,35 +1026,33 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海·二次元小偶像之夜（取消）</t>
+          <t>上海·JOing动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>东大名路638号国投大厦 音乐之门</t>
+          <t>申虹路663号 虹桥协信中心</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.11.02 13:00-11.02 19:30</t>
+          <t>2024.11.02 10:00-11.03 17:00</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>39</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>1886</v>
+      </c>
+      <c r="G15" t="n">
+        <v>65</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92591</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93044</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/gKCWSOnH1727231047223.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/GwoLrudT1728526473661.jpeg</t>
         </is>
       </c>
     </row>
@@ -1069,33 +1067,35 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第51届动漫节之音乐会篇（免费漫展）</t>
+          <t>上海·二次元小偶像之夜（取消）</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>都市路5001 上海仲盛世界商城</t>
+          <t>东大名路638号国投大厦 音乐之门</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.11.02 10:00-11.03 18:00</t>
+          <t>2024.11.02 13:00-11.02 19:30</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1048</v>
-      </c>
-      <c r="G16" t="n">
-        <v>36.9</v>
+        <v>39</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93530</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92591</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/fFFSndY41729049628568.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/gKCWSOnH1727231047223.png</t>
         </is>
       </c>
     </row>
@@ -1110,12 +1110,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·城市动漫节4th（取消）</t>
+          <t>上海·坏孩纸物语の第51届动漫节之音乐会篇（免费漫展）</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>西藏南路1号 上海大世界</t>
+          <t>都市路5001 上海仲盛世界商城</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1124,21 +1124,19 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>55</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>1049</v>
+      </c>
+      <c r="G17" t="n">
+        <v>36.9</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93341</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93530</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/cZuHHdrP1728634277406.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/fFFSndY41729049628568.jpeg</t>
         </is>
       </c>
     </row>
@@ -1153,33 +1151,35 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·恶作剧国乙＋代号鸢同人only</t>
+          <t>上海·城市动漫节4th（取消）</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
+          <t>西藏南路1号 上海大世界</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.11.02 11:00-11.02 20:30</t>
+          <t>2024.11.02 10:00-11.03 18:00</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>534</v>
-      </c>
-      <c r="G18" t="n">
-        <v>198</v>
+        <v>55</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91997</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93341</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/1Jx3TttO1725265947215.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/cZuHHdrP1728634277406.jpeg</t>
         </is>
       </c>
     </row>
@@ -1194,33 +1194,33 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·第七十六届燃梦星辰国潮国漫嘉年华-万圣狂欢-让我们在燃梦相遇吧！（免费展）</t>
+          <t>上海·恶作剧国乙＋代号鸢同人only</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>泗宝路41号 嘉宏·大橘印象荟</t>
+          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.11.02 13:00-11.03 17:00</t>
+          <t>2024.11.02 11:00-11.02 20:30</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1615</v>
+        <v>534</v>
       </c>
       <c r="G19" t="n">
-        <v>58.8</v>
+        <v>198</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91997</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/pROWU8391728382255181.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/1Jx3TttO1725265947215.jpeg</t>
         </is>
       </c>
     </row>
@@ -1230,40 +1230,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-11-02</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·恋与深空契约3.0同人Only回溯之时（取消）</t>
+          <t>上海·第七十六届燃梦星辰国潮国漫嘉年华-万圣狂欢-让我们在燃梦相遇吧！（免费展）</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>南翔镇嘉前路275号 嘉美莉雅一站式宴会中心</t>
+          <t>泗宝路41号 嘉宏·大橘印象荟</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.11.03 10:30-11.03 21:00</t>
+          <t>2024.11.02 13:00-11.03 17:00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>40</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>1615</v>
+      </c>
+      <c r="G20" t="n">
+        <v>58.8</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93449</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93173</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/e6KxRlyj1728566600416.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/pROWU8391728382255181.jpeg</t>
         </is>
       </c>
     </row>
@@ -1278,33 +1276,35 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·赤岛Trend诡影吹灯万圣鸢O</t>
+          <t>上海·恋与深空契约3.0同人Only回溯之时（取消）</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>呼兰西路123号龙盛活力小镇5号楼 摩可纳婚礼艺术中心</t>
+          <t>南翔镇嘉前路275号 嘉美莉雅一站式宴会中心</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.11.03 13:00-11.03 20:00</t>
+          <t>2024.11.03 10:30-11.03 21:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>27</v>
-      </c>
-      <c r="G21" t="n">
-        <v>168</v>
+        <v>40</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93527</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93449</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/3WMvgo481729049262603.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/e6KxRlyj1728566600416.jpeg</t>
         </is>
       </c>
     </row>
@@ -1314,38 +1314,38 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·AXG彩虹领域动漫游戏嘉年华</t>
+          <t>上海·赤岛Trend诡影吹灯万圣鸢O</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>潍坊新村街道九六广场 F2AXG彩虹岛（九六广场店）</t>
+          <t>呼兰西路123号龙盛活力小镇5号楼 摩可纳婚礼艺术中心</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.11.09 10:00-11.10 17:00</t>
+          <t>2024.11.03 13:00-11.03 20:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G22" t="n">
-        <v>58</v>
+        <v>168</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93640</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93527</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/rP8cwFGu1729664986386.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/3WMvgo481729049262603.jpeg</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·创造力动漫游戏嘉年华2.0</t>
+          <t>上海·AXG彩虹领域动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>莘福路288号 美莘商业广场</t>
+          <t>潍坊新村街道九六广场 F2AXG彩虹岛（九六广场店）</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1374,19 +1374,19 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2427</v>
+        <v>20</v>
       </c>
       <c r="G23" t="n">
-        <v>9.9</v>
+        <v>58</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92437</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93640</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/WYhzbzTu1727593484019.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/rP8cwFGu1729664986386.jpeg</t>
         </is>
       </c>
     </row>
@@ -1401,33 +1401,33 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·夜蓝诗2.0·恋与深空同人only</t>
+          <t>上海·创造力动漫游戏嘉年华2.0</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>沪闵路7388号 上海百联南方商城</t>
+          <t>莘福路288号 美莘商业广场</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.11.09 11:00-11.09 21:00</t>
+          <t>2024.11.09 10:00-11.10 17:00</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>471</v>
+        <v>2428</v>
       </c>
       <c r="G24" t="n">
-        <v>98</v>
+        <v>9.9</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93438</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92437</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/KeJJBybC1728903298004.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/WYhzbzTu1727593484019.jpeg</t>
         </is>
       </c>
     </row>
@@ -1442,33 +1442,33 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·星芒旋转 Anikura二次元派对</t>
+          <t>上海·夜蓝诗2.0·恋与深空同人only</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>沪闵路7388号 上海百联南方商城</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.11.09 14:00-11.09 17:00</t>
+          <t>2024.11.09 11:00-11.09 21:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>11</v>
+        <v>472</v>
       </c>
       <c r="G25" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93465</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93438</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/XV9uEGAz1728900548343.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/KeJJBybC1728903298004.jpeg</t>
         </is>
       </c>
     </row>
@@ -1483,33 +1483,33 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·第五人格同人Only</t>
+          <t>上海·星芒旋转 Anikura二次元派对</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.11.09 10:00-11.10 17:00</t>
+          <t>2024.11.09 14:00-11.09 17:00</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1062</v>
+        <v>11</v>
       </c>
       <c r="G26" t="n">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93718</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93465</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/4hYvCN4W1729223140208.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/XV9uEGAz1728900548343.jpeg</t>
         </is>
       </c>
     </row>
@@ -1519,38 +1519,38 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2024-11-16</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>上海·趣元界·第三届ICG动漫游戏博览会</t>
+          <t>上海·第五人格同人Only</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>西藏南路1号 上海大世界</t>
+          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>2024.11.16 10:00-11.17 17:00</t>
+          <t>2024.11.09 10:00-11.10 17:00</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>4651</v>
+        <v>1064</v>
       </c>
       <c r="G27" t="n">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92846</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93718</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/C1h14i9R1728540930986.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/4hYvCN4W1729223140208.jpeg</t>
         </is>
       </c>
     </row>
@@ -1560,38 +1560,38 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2024-11-16</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>上海·第五届长三角文博会上海国际插画艺术节</t>
+          <t>上海·趣元界·第三届ICG动漫游戏博览会</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>崧泽大道333号 国家会展中心</t>
+          <t>西藏南路1号 上海大世界</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>2024.11.22 09:00-11.25 15:00</t>
+          <t>2024.11.16 10:00-11.17 17:00</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>115</v>
+        <v>4655</v>
       </c>
       <c r="G28" t="n">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92813</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92846</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/CXUc87f81729246062802.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/C1h14i9R1728540930986.jpeg</t>
         </is>
       </c>
     </row>
@@ -1601,40 +1601,38 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2024-11-23</t>
+          <t>2024-11-22</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·ComiCon动漫展</t>
+          <t>上海·第五届长三角文博会上海国际插画艺术节</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>军工路1076号 纪希片场(秀场)</t>
+          <t>崧泽大道333号 国家会展中心</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.11.23 09:00-11.24 18:00</t>
+          <t>2024.11.22 09:00-11.25 15:00</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>14</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>115</v>
+      </c>
+      <c r="G29" t="n">
+        <v>62</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93900</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92813</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/WwDSp4971729737145743.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/CXUc87f81729246062802.jpeg</t>
         </is>
       </c>
     </row>
@@ -1649,33 +1647,35 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·cos dream country coser动漫展</t>
+          <t>上海·ComiCon动漫展</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>军工路1076号 纪希片场(秀场)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.11.23 10:00-11.24 17:00</t>
+          <t>2024.11.23 09:00-11.24 18:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>37</v>
-      </c>
-      <c r="G30" t="n">
-        <v>60</v>
+        <v>14</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93486</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93900</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/NGXdRwo21728727323251.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/WwDSp4971729737145743.png</t>
         </is>
       </c>
     </row>
@@ -1690,33 +1690,33 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·光年之外时空中的绘旅人同人ONLY</t>
+          <t>上海·cos dream country coser动漫展</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>泗泾鼓浪路220号 嘉美丽雅婚礼中心</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.11.23 10:30-11.23 21:00</t>
+          <t>2024.11.23 10:00-11.24 17:00</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>3</v>
+        <v>37</v>
       </c>
       <c r="G31" t="n">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93927</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93486</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/W7nNfX2E1729683658814.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/NGXdRwo21728727323251.jpeg</t>
         </is>
       </c>
     </row>
@@ -1731,35 +1731,33 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·第二届iPR动漫游戏嘉年华（取消）</t>
+          <t>上海·光年之外时空中的绘旅人同人ONLY</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
+          <t>泗泾鼓浪路220号 嘉美丽雅婚礼中心</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.11.23 11:00-11.24 16:00</t>
+          <t>2024.11.23 10:30-11.23 21:00</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2685</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="G32" t="n">
+        <v>98</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=90990</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93927</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/T8TJCkiA1728698774876.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/W7nNfX2E1729683658814.jpeg</t>
         </is>
       </c>
     </row>
@@ -1769,38 +1767,40 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2024-11-30</t>
+          <t>2024-11-23</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>上海·SunShine跨次元动漫游戏嘉年华2.0</t>
+          <t>上海·第二届iPR动漫游戏嘉年华（取消）</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>景泰路465号 上海园艺体验中心</t>
+          <t>盈浦街道淀山浦社区淀山湖大道851号青浦万达茂F3 万达汽车乐园(青浦万达茂店)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2024.11.30 10:30-12.01 17:00</t>
+          <t>2024.11.23 11:00-11.24 16:00</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>19</v>
-      </c>
-      <c r="G33" t="n">
-        <v>69</v>
+        <v>2685</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93445</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=90990</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/PkBLAxyI1728882644725.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/T8TJCkiA1728698774876.jpeg</t>
         </is>
       </c>
     </row>
@@ -1810,38 +1810,38 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-12-07</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·明日方舟同人ONLY</t>
+          <t>上海·SunShine跨次元动漫游戏嘉年华2.0</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>顾村镇蕰川路6号 智慧湾科创园</t>
+          <t>景泰路465号 上海园艺体验中心</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.12.07 10:00-12.07 17:00</t>
+          <t>2024.11.30 10:30-12.01 17:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>181</v>
+        <v>23</v>
       </c>
       <c r="G34" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92324</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93445</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/NgLTLVBR1725522658446.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/PkBLAxyI1728882644725.jpeg</t>
         </is>
       </c>
     </row>
@@ -1851,38 +1851,38 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-12-20</t>
+          <t>2024-12-07</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·CAFEEX咖啡节</t>
+          <t>上海·明日方舟同人ONLY</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>龙阳路2345号 上海新国际博览中心</t>
+          <t>顾村镇蕰川路6号 智慧湾科创园</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.12.20 09:30-12.22 17:30</t>
+          <t>2024.12.07 10:00-12.07 17:00</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>10</v>
+        <v>182</v>
       </c>
       <c r="G35" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93544</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92324</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/9LAP7hUC1729075059733.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/NgLTLVBR1725522658446.jpeg</t>
         </is>
       </c>
     </row>
@@ -1892,38 +1892,38 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2024-12-21</t>
+          <t>2024-12-20</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>上海·向前冲！运动番同人Only</t>
+          <t>上海·CAFEEX咖啡节</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
+          <t>龙阳路2345号 上海新国际博览中心</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2024.12.21 11:00-12.22 18:00</t>
+          <t>2024.12.20 09:30-12.22 17:30</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1252</v>
+        <v>10</v>
       </c>
       <c r="G36" t="n">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92392</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93544</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/Mvb2lCuz1728540720675.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/9LAP7hUC1729075059733.jpeg</t>
         </is>
       </c>
     </row>
@@ -1938,33 +1938,33 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>上海·旅行盛宴次元综合同人动漫节4.0·一周年庆</t>
+          <t>上海·向前冲！运动番同人Only</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>景泰路465号 上海园艺体验中心</t>
+          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2024.12.21 10:00-12.22 17:00</t>
+          <t>2024.12.21 11:00-12.22 18:00</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>6</v>
+        <v>1254</v>
       </c>
       <c r="G37" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93447</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92392</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/9uMCI2Ac1728894507590.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/Mvb2lCuz1728540720675.jpeg</t>
         </is>
       </c>
     </row>
@@ -1974,38 +1974,38 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2024-12-28</t>
+          <t>2024-12-21</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>上海·LookLook动漫嘉年华3th</t>
+          <t>上海·旅行盛宴次元综合同人动漫节4.0·一周年庆</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>曹安公路4218号 上海国际短视频中心</t>
+          <t>景泰路465号 上海园艺体验中心</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2024.12.28 10:00-12.29 17:30</t>
+          <t>2024.12.21 10:00-12.22 17:00</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1009</v>
+        <v>6</v>
       </c>
       <c r="G38" t="n">
-        <v>29.9</v>
+        <v>69</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=90495</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93447</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/DQLGW65C1726814328151.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/9uMCI2Ac1728894507590.jpeg</t>
         </is>
       </c>
     </row>
@@ -2015,36 +2015,77 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
+          <t>2024-12-28</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>上海·LookLook动漫嘉年华3th</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>曹安公路4218号 上海国际短视频中心</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2024.12.28 10:00-12.29 17:30</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1010</v>
+      </c>
+      <c r="G39" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>https://show.bilibili.com/platform/detail.html?id=90495</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/DQLGW65C1726814328151.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>2024-12-31</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>上海·星芒旋转 二次元DJ跨年派对</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>2024.12.31 18:00-2025.01.01 00:00</t>
         </is>
       </c>
-      <c r="F39" t="n">
-        <v>27</v>
-      </c>
-      <c r="G39" t="n">
+      <c r="F40" t="n">
+        <v>28</v>
+      </c>
+      <c r="G40" t="n">
         <v>70</v>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>https://show.bilibili.com/platform/detail.html?id=93489</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I40" t="inlineStr">
         <is>
           <t>//i2.hdslb.com/bfs/openplatform/202410/9u80he4k1728981349492.jpeg</t>
         </is>
@@ -2115,40 +2156,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024-10-25</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>上海·俄罗斯音乐剧《安娜·卡列尼娜》俄语巡演版</t>
+          <t>上海·【早鸟4折】“海上钢琴师”一生必听经典电影主题音乐会</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>东大名路889号 北外滩友邦大剧院</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024.10.25 19:30-10.27 16:30</t>
+          <t>2024.10.26 15:00-10.26 16:30</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>35</v>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>不可售</t>
-        </is>
+        <v>33</v>
+      </c>
+      <c r="G2" t="n">
+        <v>112</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91777</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91375</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/nu5GUuxV1725343203986.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202408/qfPgppOK1724743485013.jpeg</t>
         </is>
       </c>
     </row>
@@ -2158,38 +2197,38 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024-10-26</t>
+          <t>2024-10-27</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>上海·【早鸟4折】“海上钢琴师”一生必听经典电影主题音乐会</t>
+          <t xml:space="preserve"> 上海·【青春无限乐团】“暮光之城”“加勒比海盗”“天空之城”“自由探戈”曲目钢琴&amp;小提琴演奏烛光音乐会</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>南苏州路1247号 八号桥艺术空间</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2024.10.26 15:00-10.26 16:30</t>
+          <t>2024.10.27 13:20-11.23 20:20</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="G3" t="n">
-        <v>112</v>
+        <v>198</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91375</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92917</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202408/qfPgppOK1724743485013.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/6pu151IE1727250048973.jpeg</t>
         </is>
       </c>
     </row>
@@ -2204,33 +2243,33 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 上海·【青春无限乐团】“暮光之城”“加勒比海盗”“天空之城”“自由探戈”曲目钢琴&amp;小提琴演奏烛光音乐会</t>
+          <t>上海·次元壁击破！神级动漫金曲超燃演唱会</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>南苏州路1247号 八号桥艺术空间</t>
+          <t>王家厍路885弄云堡未来市 未来SHOW秀场</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2024.10.27 13:20-11.23 20:20</t>
+          <t>2024.10.27 19:30-10.27 21:00</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="G4" t="n">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92917</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93038</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/6pu151IE1727250048973.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/fiR1CgiJ1727418963361.jpeg</t>
         </is>
       </c>
     </row>
@@ -2245,33 +2284,33 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·次元壁击破！神级动漫金曲超燃演唱会</t>
+          <t>上海·青春无限乐团绝美炫技“双钢琴演奏"烛光音乐会流行曲目&amp;经典影视曲目对飙四手联弹</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>王家厍路885弄云堡未来市 未来SHOW秀场</t>
+          <t>南苏州路1247号 八号桥艺术空间</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024.10.27 19:30-10.27 21:00</t>
+          <t>2024.10.27 15:10-11.24 15:10</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93038</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92989</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/fiR1CgiJ1727418963361.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/sySjsTcQ1727249689293.jpeg</t>
         </is>
       </c>
     </row>
@@ -2281,38 +2320,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-10-27</t>
+          <t>2024-10-28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·青春无限乐团绝美炫技“双钢琴演奏"烛光音乐会流行曲目&amp;经典影视曲目对飙四手联弹</t>
+          <t>上海·majiko巡演-2024</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>南苏州路1247号 八号桥艺术空间</t>
+          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.10.27 15:10-11.24 15:10</t>
+          <t>2024.10.28 20:00-10.28 21:40</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>174</v>
       </c>
       <c r="G6" t="n">
-        <v>198</v>
+        <v>480</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92989</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92297</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/sySjsTcQ1727249689293.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/SuvrM0xK1726038317196.jpeg</t>
         </is>
       </c>
     </row>
@@ -2327,33 +2366,33 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·majiko巡演-2024</t>
+          <t>上海·“港乐经典·难忘金曲”纪念 陈百强·罗文 永恒典藏演唱会</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.10.28 20:00-10.28 21:40</t>
+          <t>2024.10.28 19:30-10.28 21:00</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>174</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>480</v>
+        <v>100</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92297</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93192</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/SuvrM0xK1726038317196.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/qHiHRBBn1728371444591.jpeg</t>
         </is>
       </c>
     </row>
@@ -2363,38 +2402,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-10-28</t>
+          <t>2024-10-31</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·“港乐经典·难忘金曲”纪念 陈百强·罗文 永恒典藏演唱会</t>
+          <t>上海·《夜遇外滩》首家环境式情景音乐会</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>南苏州路107号 外滩源33</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.10.28 19:30-10.28 21:00</t>
+          <t>2024.10.31 19:30-11.01 21:00</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G8" t="n">
-        <v>100</v>
+        <v>139</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93192</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93241</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/qHiHRBBn1728371444591.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/KYYiUSXk1728192323769.jpeg</t>
         </is>
       </c>
     </row>
@@ -2409,33 +2448,33 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·《夜遇外滩》首家环境式情景音乐会</t>
+          <t>上海·苏菲•珊曼妮2024巡回演唱会</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>南苏州路107号 外滩源33</t>
+          <t>重庆南路308号3楼 上海MAO LIVEHOUSE</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.10.31 19:30-11.01 21:00</t>
+          <t>2024.10.31 20:00-10.31 21:40</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G9" t="n">
-        <v>139</v>
+        <v>380</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93241</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=87918</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/KYYiUSXk1728192323769.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202406/RhhjOqDY1718160939240.jpeg</t>
         </is>
       </c>
     </row>
@@ -2445,38 +2484,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-10-31</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·苏菲•珊曼妮2024巡回演唱会</t>
+          <t>上海·Do As Infinity 2024 LIVE in SHANGHAI大无限乐团 2024演唱会</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>重庆南路308号3楼 上海MAO LIVEHOUSE</t>
+          <t>世博大道2095号4幢一层A二层 红石中心</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.10.31 20:00-10.31 21:40</t>
+          <t>2024.11.01 19:00-11.01 21:30</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>12</v>
       </c>
       <c r="G10" t="n">
-        <v>380</v>
+        <v>580</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=87918</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93302</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202406/RhhjOqDY1718160939240.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/F1kMRmQK1728632339424.jpeg</t>
         </is>
       </c>
     </row>
@@ -2491,33 +2530,33 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·Do As Infinity 2024 LIVE in SHANGHAI大无限乐团 2024演唱会</t>
+          <t>上海·“万圣节狂欢夜”流行金曲榜 经典歌曲演唱会</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>世博大道2095号4幢一层A二层 红石中心</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.11.01 19:00-11.01 21:30</t>
+          <t>2024.11.01 19:30-11.01 21:00</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
-        <v>580</v>
+        <v>100</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93302</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93404</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/F1kMRmQK1728632339424.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/ojqp6zRd1728712855902.jpeg</t>
         </is>
       </c>
     </row>
@@ -2532,12 +2571,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·“万圣节狂欢夜”流行金曲榜 经典歌曲演唱会</t>
+          <t>上海·松井祐贵 2024《阳光之旅》指弹吉他音乐会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2546,19 +2585,19 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G12" t="n">
-        <v>100</v>
+        <v>220</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93404</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92776</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/ojqp6zRd1728712855902.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/OU2qWxgM1727082424391.jpeg</t>
         </is>
       </c>
     </row>
@@ -2573,33 +2612,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·松井祐贵 2024《阳光之旅》指弹吉他音乐会</t>
+          <t>上海·混合理论——致敬林肯公园世界巡回演唱会</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心</t>
+          <t>都市路4889号（莘庄地铁站南广场） 保利上海城市剧院</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.11.01 19:30-11.01 21:00</t>
+          <t>2024.11.01 19:30-11.02 21:00</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="G13" t="n">
-        <v>220</v>
+        <v>280</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92776</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92919</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/OU2qWxgM1727082424391.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/eqQuBfcz1727246126192.jpeg</t>
         </is>
       </c>
     </row>
@@ -2614,33 +2653,33 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·混合理论——致敬林肯公园世界巡回演唱会</t>
+          <t>宝山·『LiveROX!次元音乐派对』幻夜续章｜二次元ACG音乐会</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>都市路4889号（莘庄地铁站南广场） 保利上海城市剧院</t>
+          <t>蕴川路6号智慧湾科创园17号楼 智慧湾艺术中心</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.11.01 19:30-11.02 21:00</t>
+          <t>2024.11.01 20:00-11.01 22:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G14" t="n">
-        <v>280</v>
+        <v>100</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92919</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93088</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/eqQuBfcz1727246126192.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/Wac6ajnr1728461206759.png</t>
         </is>
       </c>
     </row>
@@ -2650,38 +2689,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-11-01</t>
+          <t>2024-11-02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>宝山·『LiveROX!次元音乐派对』幻夜续章｜二次元ACG音乐会</t>
+          <t>上海·欢迎来到绵羊咖啡屋! 中国第二回 仲村宗悟 梶原岳人</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>蕴川路6号智慧湾科创园17号楼 智慧湾艺术中心</t>
+          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.11.01 20:00-11.01 22:00</t>
+          <t>2024.11.02 12:00-11.02 21:30</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>30</v>
+        <v>97</v>
       </c>
       <c r="G15" t="n">
-        <v>100</v>
+        <v>380</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93088</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91176</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/Wac6ajnr1728461206759.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202408/QtV99HO81724384169942.jpeg</t>
         </is>
       </c>
     </row>
@@ -2696,33 +2735,33 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·欢迎来到绵羊咖啡屋! 中国第二回 仲村宗悟 梶原岳人</t>
+          <t>上海·青春无限乐团钢琴独奏&amp;芭蕾舞表演梦幻联动表演经典影视作品曲目</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>茂名南路57号近长乐路 上海兰心大戏院</t>
+          <t>南苏州路1247号 八号桥艺术空间</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.11.02 12:00-11.02 21:30</t>
+          <t>2024.11.02 15:00-11.24 17:10</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>97</v>
+        <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>380</v>
+        <v>238</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91176</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92988</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202408/QtV99HO81724384169942.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/wmizsXC21727418983817.png</t>
         </is>
       </c>
     </row>
@@ -2732,38 +2771,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·青春无限乐团钢琴独奏&amp;芭蕾舞表演梦幻联动表演经典影视作品曲目</t>
+          <t>上海·「多厨狂喜」白金交响乐团二次元交响音乐会</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>南苏州路1247号 八号桥艺术空间</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.11.02 15:00-11.24 17:10</t>
+          <t>2024.11.03 14:00-11.03 16:00</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>195</v>
       </c>
       <c r="G17" t="n">
-        <v>238</v>
+        <v>188</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92988</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93086</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/wmizsXC21727418983817.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/GvAAxiwb1727619935967.jpeg</t>
         </is>
       </c>
     </row>
@@ -2778,33 +2817,33 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海·「多厨狂喜」白金交响乐团二次元交响音乐会</t>
+          <t>上海·司南2024「出发」个人首巡最终场</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
+          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.11.03 14:00-11.03 16:00</t>
+          <t>2024.11.03 19:30-11.03 21:30</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>194</v>
+        <v>19</v>
       </c>
       <c r="G18" t="n">
-        <v>188</v>
+        <v>149.5</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93086</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92942</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/GvAAxiwb1727619935967.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/voxVudGs1727331756649.jpeg</t>
         </is>
       </c>
     </row>
@@ -2814,38 +2853,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-11-03</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·司南2024「出发」个人首巡最终场</t>
+          <t>上海·2024年刘明月专场生日会</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.11.03 19:30-11.03 21:30</t>
+          <t>2024.11.09 11:11-11.09 12:30</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>19</v>
+        <v>202</v>
       </c>
       <c r="G19" t="n">
-        <v>149.5</v>
+        <v>399</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92942</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93079</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/voxVudGs1727331756649.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/lgdmiGF21727487105022.png</t>
         </is>
       </c>
     </row>
@@ -2860,33 +2899,33 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·2024年刘明月专场生日会</t>
+          <t>上海·【大乐】《怦然心动·爱乐之城》奥斯卡之夜影视金曲视听音乐会</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.11.09 11:11-11.09 12:30</t>
+          <t>2024.11.09 19:30-11.09 21:00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>202</v>
+        <v>3</v>
       </c>
       <c r="G20" t="n">
-        <v>399</v>
+        <v>50</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93079</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93082</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/lgdmiGF21727487105022.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/HLyh2lMk1727601687746.jpeg</t>
         </is>
       </c>
     </row>
@@ -2901,7 +2940,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>上海·【大乐】《怦然心动·爱乐之城》奥斯卡之夜影视金曲视听音乐会</t>
+          <t>上海·【大乐】【亲子合家欢】《我的邻居龙猫》宫崎骏·久石让动漫作品音乐会</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2911,23 +2950,23 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.11.09 19:30-11.09 21:00</t>
+          <t>2024.11.09 15:00-11.09 16:30</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G21" t="n">
         <v>50</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93082</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93077</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/HLyh2lMk1727601687746.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/IH31eXGt1727668337378.jpeg</t>
         </is>
       </c>
     </row>
@@ -2942,33 +2981,33 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·【大乐】【亲子合家欢】《我的邻居龙猫》宫崎骏·久石让动漫作品音乐会</t>
+          <t>上海·早鸟7折天空之城—久石让·宫崎骏动漫视听轻音乐之旅钢琴音乐会</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>张杨路400号 兰馨悦立方</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.11.09 15:00-11.09 16:30</t>
+          <t>2024.11.09 14:30-11.09 16:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G22" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93077</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92887</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/IH31eXGt1727668337378.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/uwAkpsXa1727237901794.jpeg</t>
         </is>
       </c>
     </row>
@@ -2983,7 +3022,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·早鸟7折天空之城—久石让·宫崎骏动漫视听轻音乐之旅钢琴音乐会</t>
+          <t>上海·早鸟7折菊次郎的夏天—久石让轻音乐之旅钢琴音乐会</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2993,23 +3032,23 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.11.09 14:30-11.09 16:00</t>
+          <t>2024.11.09 19:30-11.09 21:00</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="G23" t="n">
         <v>70</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92887</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92876</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/uwAkpsXa1727237901794.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/QiRW70mZ1727238565641.jpeg</t>
         </is>
       </c>
     </row>
@@ -3019,38 +3058,40 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2024-11-09</t>
+          <t>2024-11-10</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·早鸟7折菊次郎的夏天—久石让轻音乐之旅钢琴音乐会</t>
+          <t>上海·【漫乐季】《冠位时之门：闪耀UP》Fun肆二次元·动漫ACG超燃音乐盛典2024（取消）</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>张杨路400号 兰馨悦立方</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.11.09 19:30-11.09 21:00</t>
+          <t>2024.11.10 14:00-11.10 15:30</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
-      </c>
-      <c r="G24" t="n">
-        <v>70</v>
+        <v>71</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>不可售</t>
+        </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92876</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92564</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/QiRW70mZ1727238565641.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/lq8ZrNwk1726622482193.jpeg</t>
         </is>
       </c>
     </row>
@@ -3161,7 +3202,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G27" t="n">
         <v>266</v>
@@ -3735,10 +3776,10 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G41" t="n">
-        <v>180</v>
+        <v>280</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -4163,7 +4204,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
       <c r="G2" t="n">
         <v>20</v>
@@ -4413,7 +4454,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G8" t="n">
         <v>30</v>
@@ -4454,7 +4495,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3135</v>
+        <v>3137</v>
       </c>
       <c r="G9" t="n">
         <v>30</v>
@@ -4495,7 +4536,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="G10" t="n">
         <v>10</v>
@@ -4536,7 +4577,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>910</v>
+        <v>913</v>
       </c>
       <c r="G11" t="n">
         <v>30</v>
@@ -4741,7 +4782,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="G16" t="n">
         <v>30</v>
@@ -4768,7 +4809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4822,38 +4863,38 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2024-07-26</t>
+          <t>2024-09-09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>上海·盗墓笔记官方授权「四季同书」主题店</t>
+          <t>上海·日漫咖啡体验</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>南京东路830号第一百货商业中心B馆5楼(海底捞旁边) 第一百货商业中心</t>
+          <t>虹桥路1438号高岛屋百货6楼 Oasis漫画喫茶</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2024.07.26 00:00-11.03 23:59</t>
+          <t>2024.09.09 10:00-12.31 22:00</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2574</v>
+        <v>177</v>
       </c>
       <c r="G2" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=89200</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91993</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202407/b4w7Ifkm1720766324652.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/IV5rInWT1725347808557.jpeg</t>
         </is>
       </c>
     </row>
@@ -4863,38 +4904,38 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2024-09-09</t>
+          <t>2024-09-26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>上海·日漫咖啡体验</t>
+          <t>上海·【神秘的西夏陵】大空间高沉浸探险体验</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>虹桥路1438号高岛屋百货6楼 Oasis漫画喫茶</t>
+          <t>南京西路325号 上海市历史博物馆</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2024.09.09 10:00-12.31 22:00</t>
+          <t>2024.09.26 10:00-12.31 19:00</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>177</v>
+        <v>38</v>
       </c>
       <c r="G3" t="n">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91993</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92581</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/IV5rInWT1725347808557.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/jeDZO2cS1726302714881.jpeg</t>
         </is>
       </c>
     </row>
@@ -4904,38 +4945,38 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2024-09-15</t>
+          <t>2024-09-28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>上海 洛天依歌行宇宙·无限遨游 沉浸式体验展</t>
+          <t>上海·［咒术回战 2024 剧场版 咒术回战 0］主题咖啡厅</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>中山北路3300号 上海月星环球港</t>
+          <t>大悦城 次元波板糖</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2024.09.15 10:00-10.31 22:00</t>
+          <t>2024.09.28 00:00-10.27 23:59</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2511</v>
+        <v>417</v>
       </c>
       <c r="G4" t="n">
-        <v>138</v>
+        <v>30</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91175</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92608</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202408/ei9COXS41724405861343.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/DBTiL9sY1726727259104.png</t>
         </is>
       </c>
     </row>
@@ -4945,38 +4986,38 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2024-09-26</t>
+          <t>2024-10-01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>上海·【神秘的西夏陵】大空间高沉浸探险体验</t>
+          <t>上海·三丽鸥家族Sanrio Characters主题餐厅·海滩奇遇季</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>南京西路325号 上海市历史博物馆</t>
+          <t>南京东路800号4楼 上海市第一百货商店-C馆</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2024.09.26 10:00-12.31 19:00</t>
+          <t>2024.10.01 00:00-11.19 23:59</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>38</v>
+        <v>642</v>
       </c>
       <c r="G5" t="n">
-        <v>108</v>
+        <v>10</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92581</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93078</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/jeDZO2cS1726302714881.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/aiu4g5K21727677592777.png</t>
         </is>
       </c>
     </row>
@@ -4986,38 +5027,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2024-09-28</t>
+          <t>2024-10-10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>上海·［咒术回战 2024 剧场版 咒术回战 0］主题咖啡厅</t>
+          <t>上海·「火影忍者疾风传 × animate cafe」</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>大悦城 次元波板糖</t>
+          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2024.09.28 00:00-10.27 23:59</t>
+          <t>2024.10.10 00:00-11.12 23:59</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>416</v>
+        <v>913</v>
       </c>
       <c r="G6" t="n">
         <v>30</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92608</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92883</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/DBTiL9sY1726727259104.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/aQIhaIgt1727249498713.png</t>
         </is>
       </c>
     </row>
@@ -5027,38 +5068,38 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2024-10-18</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>上海·2024·《世界之外》x  萌果酱谷子咖啡</t>
+          <t>上海·幻境尘影—无期迷途光影展</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>南京东路340号百联ZX 萌果酱谷子咖啡（百联）</t>
+          <t>陆家嘴西路168号 上海正大广场</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2024.10.01 00:00-12.11 23:59</t>
+          <t>2024.10.18 00:00-11.30 23:59</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3135</v>
+        <v>1979</v>
       </c>
       <c r="G7" t="n">
-        <v>30</v>
+        <v>98</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93006</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93269</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/qtffZOKB1727426243733.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/kq6Pmpkv1728728206204.png</t>
         </is>
       </c>
     </row>
@@ -5068,38 +5109,38 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-10-01</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>上海·三丽鸥家族Sanrio Characters主题餐厅·海滩奇遇季</t>
+          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·场贩</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>南京东路800号4楼 上海市第一百货商店-C馆</t>
+          <t>中山北路3300号 上海月星环球港</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2024.10.01 00:00-11.19 23:59</t>
+          <t>2024.10.26 00:00-11.24 23:59</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>640</v>
+        <v>48</v>
       </c>
       <c r="G8" t="n">
         <v>10</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93078</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93600</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/aiu4g5K21727677592777.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/SJdbDqYE1729147018420.png</t>
         </is>
       </c>
     </row>
@@ -5109,38 +5150,38 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2024-10-10</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>上海·「火影忍者疾风传 × animate cafe」</t>
+          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·场贩</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
+          <t>中山北路3300号 上海月星环球港</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2024.10.10 00:00-11.12 23:59</t>
+          <t>2024.10.26 00:00-11.24 23:59</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>910</v>
+        <v>48</v>
       </c>
       <c r="G9" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92883</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93600</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/aQIhaIgt1727249498713.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/SJdbDqYE1729147018420.png</t>
         </is>
       </c>
     </row>
@@ -5150,38 +5191,38 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2024-10-17</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>上海·蜡笔小新：我们的恐龙日记x HAPPY ZOO 主题咖啡厅</t>
+          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·餐饮</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>南京东路340号百联zx创趣场四楼05号 HAPPY ZOO</t>
+          <t>中山北路3300号 上海月星环球港</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2024.10.17 00:00-10.27 23:59</t>
+          <t>2024.10.26 00:00-11.24 23:59</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>330</v>
+        <v>75</v>
       </c>
       <c r="G10" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93221</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93578</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/nzGP5KRA1728526131597.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/NAELHmKL1729145655311.png</t>
         </is>
       </c>
     </row>
@@ -5191,38 +5232,38 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2024-10-18</t>
+          <t>2024-10-26</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>上海·幻境尘影—无期迷途光影展</t>
+          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·餐饮</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>陆家嘴西路168号 上海正大广场</t>
+          <t>中山北路3300号 上海月星环球港</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2024.10.18 00:00-11.30 23:59</t>
+          <t>2024.10.26 00:00-11.24 23:59</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1976</v>
+        <v>75</v>
       </c>
       <c r="G11" t="n">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93269</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93578</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/kq6Pmpkv1728728206204.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/NAELHmKL1729145655311.png</t>
         </is>
       </c>
     </row>
@@ -5237,33 +5278,33 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·场贩</t>
+          <t>上海·【早鸟4折】“海上钢琴师”一生必听经典电影主题音乐会</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>中山北路3300号 上海月星环球港</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2024.10.26 00:00-11.24 23:59</t>
+          <t>2024.10.26 15:00-10.26 16:30</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="G12" t="n">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93600</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91375</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/SJdbDqYE1729147018420.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202408/qfPgppOK1724743485013.jpeg</t>
         </is>
       </c>
     </row>
@@ -5278,33 +5319,33 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·场贩</t>
+          <t>上海·杜莎夫人蜡像馆万圣节奇妙周x次元动漫嘉年华</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>中山北路3300号 上海月星环球港</t>
+          <t>南京西路新世界商厦10层 上海杜莎夫人蜡像馆</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2024.10.26 00:00-11.24 23:59</t>
+          <t>2024.10.26 16:00-11.01 21:00</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>48</v>
+        <v>8</v>
       </c>
       <c r="G13" t="n">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93600</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93728</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/SJdbDqYE1729147018420.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/DzsWUuCu1729479657498.jpeg</t>
         </is>
       </c>
     </row>
@@ -5314,38 +5355,38 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2024-10-26</t>
+          <t>2024-10-27</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·餐饮</t>
+          <t>上海·“VWonderland万圣派对”虚拟主播见面会</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>中山北路3300号 上海月星环球港</t>
+          <t>苏虹路266号 魔法魅影•沉浸式Live剧场</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>2024.10.26 00:00-11.24 23:59</t>
+          <t>2024.10.27 10:00-10.27 22:00</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="G14" t="n">
         <v>30</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93578</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93298</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/NAELHmKL1729145655311.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/Dh8Mytgq1728637643173.png</t>
         </is>
       </c>
     </row>
@@ -5355,38 +5396,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2024-10-26</t>
+          <t>2024-10-27</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>上海·NIJISANJI EN X KAKACODE主题快闪店·餐饮</t>
+          <t>上海·次元壁击破！神级动漫金曲超燃演唱会</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>中山北路3300号 上海月星环球港</t>
+          <t>王家厍路885弄云堡未来市 未来SHOW秀场</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>2024.10.26 00:00-11.24 23:59</t>
+          <t>2024.10.27 19:30-10.27 21:00</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="G15" t="n">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93578</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93038</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/NAELHmKL1729145655311.png</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/fiR1CgiJ1727418963361.jpeg</t>
         </is>
       </c>
     </row>
@@ -5396,38 +5437,38 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2024-10-27</t>
+          <t>2024-10-28</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>上海·“VWonderland万圣派对”虚拟主播见面会</t>
+          <t>上海·蜡笔小新：我们的恐龙日记x HAPPY ZOO 主题咖啡厅</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>苏虹路266号 魔法魅影•沉浸式Live剧场</t>
+          <t>南京东路340号百联zx创趣场四楼05号 HAPPY ZOO</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>2024.10.27 10:00-10.27 22:00</t>
+          <t>2024.10.28 00:00-11.10 23:59</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G16" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93298</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93719</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/Dh8Mytgq1728637643173.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/zhKQZnHB1729477411932.png</t>
         </is>
       </c>
     </row>
@@ -5437,38 +5478,38 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2024-10-28</t>
+          <t>2024-10-31</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>上海·蜡笔小新：我们的恐龙日记x HAPPY ZOO 主题咖啡厅</t>
+          <t>上海 ·《天官赐福》动画四周年纪念展</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>南京东路340号百联zx创趣场四楼05号 HAPPY ZOO</t>
+          <t>南京西路2-68号 上海新世界城</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>2024.10.28 00:00-11.10 23:59</t>
+          <t>2024.10.31 00:00-11.30 23:59</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>20</v>
+        <v>1866</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>9.9</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93719</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92995</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/zhKQZnHB1729477411932.png</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/BJWdBkrc1727422599776.jpeg</t>
         </is>
       </c>
     </row>
@@ -5483,33 +5524,33 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>上海 ·《天官赐福》动画四周年纪念展</t>
+          <t>上海·JinkyHuang x Hello Kitty 「柘柘之境」</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>南京西路2-68号 上海新世界城</t>
+          <t>淮海中路523号TX淮海F2层 BIP.Gallery</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2024.10.31 00:00-11.30 23:59</t>
+          <t>2024.10.31 11:00-2025.02.28 21:00</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1860</v>
+        <v>6</v>
       </c>
       <c r="G18" t="n">
-        <v>9.9</v>
+        <v>68</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92995</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93594</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/BJWdBkrc1727422599776.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/uIC27Eyw1729150170638.jpeg</t>
         </is>
       </c>
     </row>
@@ -5519,38 +5560,38 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2024-10-31</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>上海·JinkyHuang x Hello Kitty 「柘柘之境」</t>
+          <t>上海·“万圣节狂欢夜”流行金曲榜 经典歌曲演唱会</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>淮海中路523号TX淮海F2层 BIP.Gallery</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>2024.10.31 11:00-2025.02.28 21:00</t>
+          <t>2024.11.01 19:30-11.01 21:00</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G19" t="n">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93594</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93404</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/uIC27Eyw1729150170638.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/ojqp6zRd1728712855902.jpeg</t>
         </is>
       </c>
     </row>
@@ -5560,38 +5601,38 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2024-10-31</t>
+          <t>2024-11-01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>上海·苏菲•珊曼妮2024巡回演唱会</t>
+          <t>宝山·『LiveROX!次元音乐派对』幻夜续章｜二次元ACG音乐会</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>重庆南路308号3楼 上海MAO LIVEHOUSE</t>
+          <t>蕴川路6号智慧湾科创园17号楼 智慧湾艺术中心</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>2024.10.31 20:00-10.31 21:40</t>
+          <t>2024.11.01 20:00-11.01 22:00</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="G20" t="n">
-        <v>380</v>
+        <v>100</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=87918</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93088</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202406/RhhjOqDY1718160939240.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/Wac6ajnr1728461206759.png</t>
         </is>
       </c>
     </row>
@@ -5601,38 +5642,38 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2024-11-01</t>
+          <t>2024-11-02</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>宝山·『LiveROX!次元音乐派对』幻夜续章｜二次元ACG音乐会</t>
+          <t>上海·JOing动漫游戏嘉年华</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>蕴川路6号智慧湾科创园17号楼 智慧湾艺术中心</t>
+          <t>申虹路663号 虹桥协信中心</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2024.11.01 20:00-11.01 22:00</t>
+          <t>2024.11.02 10:00-11.03 17:00</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>30</v>
+        <v>1886</v>
       </c>
       <c r="G21" t="n">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93088</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93044</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/Wac6ajnr1728461206759.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/GwoLrudT1728526473661.jpeg</t>
         </is>
       </c>
     </row>
@@ -5647,33 +5688,33 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>上海·JOing动漫游戏嘉年华</t>
+          <t>上海·坏孩纸物语の第51届动漫节之音乐会篇（免费漫展）</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>申虹路663号 虹桥协信中心</t>
+          <t>都市路5001 上海仲盛世界商城</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2024.11.02 10:00-11.03 17:00</t>
+          <t>2024.11.02 10:00-11.03 18:00</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1884</v>
+        <v>1049</v>
       </c>
       <c r="G22" t="n">
-        <v>65</v>
+        <v>36.9</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93044</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93530</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/GwoLrudT1728526473661.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/fFFSndY41729049628568.jpeg</t>
         </is>
       </c>
     </row>
@@ -5688,33 +5729,33 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>上海·坏孩纸物语の第51届动漫节之音乐会篇（免费漫展）</t>
+          <t>上海·恶作剧国乙＋代号鸢同人only</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>都市路5001 上海仲盛世界商城</t>
+          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2024.11.02 10:00-11.03 18:00</t>
+          <t>2024.11.02 11:00-11.02 20:30</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1048</v>
+        <v>534</v>
       </c>
       <c r="G23" t="n">
-        <v>36.9</v>
+        <v>198</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93530</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91997</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/fFFSndY41729049628568.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/1Jx3TttO1725265947215.jpeg</t>
         </is>
       </c>
     </row>
@@ -5729,33 +5770,33 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>上海·恶作剧国乙＋代号鸢同人only</t>
+          <t>上海·青春无限乐团钢琴独奏&amp;芭蕾舞表演梦幻联动表演经典影视作品曲目</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>政通路189号五角场万达广场C栋 元气森林livehouse</t>
+          <t>南苏州路1247号 八号桥艺术空间</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2024.11.02 11:00-11.02 20:30</t>
+          <t>2024.11.02 15:00-11.24 17:10</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>534</v>
+        <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91997</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92988</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/1Jx3TttO1725265947215.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/wmizsXC21727418983817.png</t>
         </is>
       </c>
     </row>
@@ -5765,38 +5806,38 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>上海·第七十六届燃梦星辰国潮国漫嘉年华-万圣狂欢-让我们在燃梦相遇吧！（免费展）</t>
+          <t>上海·「多厨狂喜」白金交响乐团二次元交响音乐会</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>泗宝路41号 嘉宏·大橘印象荟</t>
+          <t>丁香路425号(上海科技馆地铁站1号口步行460米) 上海东方艺术中心音乐厅</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2024.11.02 13:00-11.03 17:00</t>
+          <t>2024.11.03 14:00-11.03 16:00</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1615</v>
+        <v>195</v>
       </c>
       <c r="G25" t="n">
-        <v>58.8</v>
+        <v>188</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93173</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93086</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/pROWU8391728382255181.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/GvAAxiwb1727619935967.jpeg</t>
         </is>
       </c>
     </row>
@@ -5806,38 +5847,38 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2024-11-02</t>
+          <t>2024-11-03</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>上海·青春无限乐团钢琴独奏&amp;芭蕾舞表演梦幻联动表演经典影视作品曲目</t>
+          <t>上海·司南2024「出发」个人首巡最终场</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>南苏州路1247号 八号桥艺术空间</t>
+          <t>嘉兴路街道瑞虹路188号瑞虹天地月亮湾3层 Modern Sky LAB摩登天空(瑞虹天地店)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2024.11.02 15:00-11.24 17:10</t>
+          <t>2024.11.03 19:30-11.03 21:30</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="G26" t="n">
-        <v>238</v>
+        <v>149.5</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92988</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92942</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/wmizsXC21727418983817.png</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/voxVudGs1727331756649.jpeg</t>
         </is>
       </c>
     </row>
@@ -5934,33 +5975,33 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>上海·【大乐】《怦然心动·爱乐之城》奥斯卡之夜影视金曲视听音乐会</t>
+          <t>上海·2024年刘明月专场生日会</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>虹许路731号4号楼 THE BOXX•城市乐园</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>2024.11.09 19:30-11.09 21:00</t>
+          <t>2024.11.09 11:11-11.09 12:30</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>3</v>
+        <v>202</v>
       </c>
       <c r="G29" t="n">
-        <v>50</v>
+        <v>399</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93082</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93079</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/HLyh2lMk1727601687746.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/lgdmiGF21727487105022.png</t>
         </is>
       </c>
     </row>
@@ -5975,33 +6016,33 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>上海·创造力动漫游戏嘉年华2.0</t>
+          <t>上海·【大乐】《怦然心动·爱乐之城》奥斯卡之夜影视金曲视听音乐会</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>莘福路288号 美莘商业广场</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>2024.11.09 10:00-11.10 17:00</t>
+          <t>2024.11.09 19:30-11.09 21:00</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2427</v>
+        <v>3</v>
       </c>
       <c r="G30" t="n">
-        <v>9.9</v>
+        <v>50</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92437</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93082</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/WYhzbzTu1727593484019.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/HLyh2lMk1727601687746.jpeg</t>
         </is>
       </c>
     </row>
@@ -6016,33 +6057,33 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>上海·夜蓝诗2.0·恋与深空同人only</t>
+          <t>上海·【大乐】【亲子合家欢】《我的邻居龙猫》宫崎骏·久石让动漫作品音乐会</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>沪闵路7388号 上海百联南方商城</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>2024.11.09 11:00-11.09 21:00</t>
+          <t>2024.11.09 15:00-11.09 16:30</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>471</v>
+        <v>7</v>
       </c>
       <c r="G31" t="n">
-        <v>98</v>
+        <v>50</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93438</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93077</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/KeJJBybC1728903298004.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202409/IH31eXGt1727668337378.jpeg</t>
         </is>
       </c>
     </row>
@@ -6057,33 +6098,33 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>上海·星芒旋转 Anikura二次元派对</t>
+          <t>上海·创造力动漫游戏嘉年华2.0</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>莘福路288号 美莘商业广场</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>2024.11.09 14:00-11.09 17:00</t>
+          <t>2024.11.09 10:00-11.10 17:00</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>11</v>
+        <v>2428</v>
       </c>
       <c r="G32" t="n">
-        <v>60</v>
+        <v>9.9</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93465</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92437</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/XV9uEGAz1728900548343.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202409/WYhzbzTu1727593484019.jpeg</t>
         </is>
       </c>
     </row>
@@ -6098,33 +6139,33 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>上海·第五人格同人Only</t>
+          <t>上海·夜蓝诗2.0·恋与深空同人only</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
+          <t>沪闵路7388号 上海百联南方商城</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>2024.11.09 10:00-11.10 17:00</t>
+          <t>2024.11.09 11:00-11.09 21:00</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1062</v>
+        <v>472</v>
       </c>
       <c r="G33" t="n">
-        <v>68</v>
+        <v>98</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93718</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93438</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/4hYvCN4W1729223140208.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/KeJJBybC1728903298004.jpeg</t>
         </is>
       </c>
     </row>
@@ -6134,38 +6175,38 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>上海·“法国姐姐”乔伊丝·乔纳森《小意思》</t>
+          <t>上海·星芒旋转 Anikura二次元派对</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>高青西路777号 上海前滩31演艺中心</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>2024.11.15 19:30-11.15 21:00</t>
+          <t>2024.11.09 14:00-11.09 17:00</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G34" t="n">
-        <v>280</v>
+        <v>60</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91619</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93465</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202408/VnZEk71H1725014748758.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/XV9uEGAz1728900548343.jpeg</t>
         </is>
       </c>
     </row>
@@ -6175,38 +6216,38 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2024-11-15</t>
+          <t>2024-11-09</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>上海·「WIND BREAKER × animate cafe」</t>
+          <t>上海·第五人格同人Only</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
+          <t>金陵东路500号(大世界地铁站6号口步行60米) 亚龙国际广场</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2024.11.15 00:00-12.15 23:59</t>
+          <t>2024.11.09 10:00-11.10 17:00</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>329</v>
+        <v>1064</v>
       </c>
       <c r="G35" t="n">
-        <v>30</v>
+        <v>68</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93422</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93718</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/TGPx1EZW1728892799830.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/4hYvCN4W1729223140208.jpeg</t>
         </is>
       </c>
     </row>
@@ -6216,12 +6257,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>2024-11-16</t>
+          <t>2024-11-15</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>上海·变形金刚音乐会40周年特别版</t>
+          <t>上海·“法国姐姐”乔伊丝·乔纳森《小意思》</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6231,23 +6272,23 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2024.11.16 19:30-11.16 21:30</t>
+          <t>2024.11.15 19:30-11.15 21:00</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="G36" t="n">
-        <v>266</v>
+        <v>280</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=90031</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=91619</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/5zTUqO9f1727061199503.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202408/VnZEk71H1725014748758.jpeg</t>
         </is>
       </c>
     </row>
@@ -6257,38 +6298,38 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>2024-11-16</t>
+          <t>2024-11-15</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>上海·趣元界·第三届ICG动漫游戏博览会</t>
+          <t>上海·「WIND BREAKER × animate cafe」</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>西藏南路1号 上海大世界</t>
+          <t>西藏北路198号大悦城北座8楼N809-1 animate cafe上海店</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2024.11.16 10:00-11.17 17:00</t>
+          <t>2024.11.15 00:00-12.15 23:59</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4651</v>
+        <v>331</v>
       </c>
       <c r="G37" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92846</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93422</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/C1h14i9R1728540930986.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/TGPx1EZW1728892799830.jpeg</t>
         </is>
       </c>
     </row>
@@ -6298,38 +6339,38 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2024-11-23</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>上海·杨丽萍作品 2022版舞剧《孔雀》</t>
+          <t>上海·Ayasa LIVE TOUR 2024〜D.D.D.〜</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>东大名路889号 北外滩友邦大剧院</t>
+          <t>宜昌路179号 万代南梦宫上海文化中心-梦想剧场</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2024.11.22 19:30-11.24 17:00</t>
+          <t>2024.11.23 14:30-11.23 16:00</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>16</v>
+        <v>489</v>
       </c>
       <c r="G38" t="n">
-        <v>880</v>
+        <v>380</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=91785</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=92891</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202409/PsSuiyCu1725341943682.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/FQDXXgRQ1727260682840.jpeg</t>
         </is>
       </c>
     </row>
@@ -6339,38 +6380,38 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2024-11-22</t>
+          <t>2024-11-23</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>上海·第五届长三角文博会上海国际插画艺术节</t>
+          <t>上海·cos dream country coser动漫展</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>崧泽大道333号 国家会展中心</t>
+          <t>海潮路133号B1 JUMP工坊</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2024.11.22 09:00-11.25 15:00</t>
+          <t>2024.11.23 10:00-11.24 17:00</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>115</v>
+        <v>37</v>
       </c>
       <c r="G39" t="n">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92813</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93486</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202410/CXUc87f81729246062802.jpeg</t>
+          <t>//i1.hdslb.com/bfs/openplatform/202410/NGXdRwo21728727323251.jpeg</t>
         </is>
       </c>
     </row>
@@ -6385,33 +6426,33 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>上海·Ayasa LIVE TOUR 2024〜D.D.D.〜</t>
+          <t>上海·光年之外时空中的绘旅人同人ONLY</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>宜昌路179号 万代南梦宫上海文化中心-梦想剧场</t>
+          <t>泗泾鼓浪路220号 嘉美丽雅婚礼中心</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2024.11.23 14:30-11.23 16:00</t>
+          <t>2024.11.23 10:30-11.23 21:00</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>489</v>
+        <v>4</v>
       </c>
       <c r="G40" t="n">
-        <v>380</v>
+        <v>98</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92891</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93927</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/FQDXXgRQ1727260682840.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/W7nNfX2E1729683658814.jpeg</t>
         </is>
       </c>
     </row>
@@ -6421,38 +6462,38 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2024-11-23</t>
+          <t>2024-11-27</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>上海·cos dream country coser动漫展</t>
+          <t>上海·“Hey jude”致敬The Beatles披头士乐队金曲演唱会</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>海潮路133号B1 JUMP工坊</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2024.11.23 10:00-11.24 17:00</t>
+          <t>2024.11.27 19:30-11.27 21:00</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="G41" t="n">
-        <v>60</v>
+        <v>90</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93486</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93193</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202410/NGXdRwo21728727323251.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/JLFmOTIa1728464039896.jpeg</t>
         </is>
       </c>
     </row>
@@ -6462,38 +6503,38 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2024-12-06</t>
+          <t>2024-11-30</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>上海·正版国漫 首部2.5次元舞台剧《狐妖小红娘》全国首演</t>
+          <t>上海·SunShine跨次元动漫游戏嘉年华2.0</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>上海市徐汇区中山南二路859号 宛平剧院-大剧场</t>
+          <t>景泰路465号 上海园艺体验中心</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2024.12.06 19:30-12.07 21:30</t>
+          <t>2024.11.30 10:30-12.01 17:00</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="G42" t="n">
-        <v>180</v>
+        <v>69</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93365</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93445</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>//i0.hdslb.com/bfs/openplatform/202410/ZAMEOQvC1728712385953.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202410/PkBLAxyI1728882644725.jpeg</t>
         </is>
       </c>
     </row>
@@ -6503,38 +6544,38 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2024-12-07</t>
+          <t>2024-12-06</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>上海·【大乐】《卡农Canon in D》世界经典作品音乐会</t>
+          <t>上海·正版国漫 首部2.5次元舞台剧《狐妖小红娘》全国首演</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>南京西路1376号 上海商城剧院</t>
+          <t>上海市徐汇区中山南二路859号 宛平剧院-大剧场</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2024.12.07 19:30-12.07 21:00</t>
+          <t>2024.12.06 19:30-12.07 21:30</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="G43" t="n">
-        <v>50</v>
+        <v>180</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=93081</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93365</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>//i2.hdslb.com/bfs/openplatform/202409/oDbouDQO1727599939832.jpeg</t>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/ZAMEOQvC1728712385953.jpeg</t>
         </is>
       </c>
     </row>
@@ -6549,33 +6590,33 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>上海·明日方舟同人ONLY</t>
+          <t>上海·【大乐】《卡农Canon in D》世界经典作品音乐会</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>顾村镇蕰川路6号 智慧湾科创园</t>
+          <t>南京西路1376号 上海商城剧院</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2024.12.07 10:00-12.07 17:00</t>
+          <t>2024.12.07 19:30-12.07 21:00</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>181</v>
+        <v>9</v>
       </c>
       <c r="G44" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>https://show.bilibili.com/platform/detail.html?id=92324</t>
+          <t>https://show.bilibili.com/platform/detail.html?id=93081</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>//i1.hdslb.com/bfs/openplatform/202409/NgLTLVBR1725522658446.jpeg</t>
+          <t>//i2.hdslb.com/bfs/openplatform/202409/oDbouDQO1727599939832.jpeg</t>
         </is>
       </c>
     </row>
@@ -6604,10 +6645,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G45" t="n">
-        <v>180</v>
+        <v>280</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -6727,7 +6768,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1252</v>
+        <v>1254</v>
       </c>
       <c r="G48" t="n">
         <v>68</v>
@@ -6850,7 +6891,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="G51" t="n">
         <v>29.9</v>
@@ -6891,7 +6932,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G52" t="n">
         <v>70</v>
@@ -6904,6 +6945,47 @@
       <c r="I52" t="inlineStr">
         <is>
           <t>//i2.hdslb.com/bfs/openplatform/202410/9u80he4k1728981349492.jpeg</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>上海·俄罗斯国家古典芭蕾剧院《天鹅湖》</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>都市路4889号（莘庄地铁站南广场） 保利上海城市剧院</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2025.01.01 15:00-01.01 21:30</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="n">
+        <v>126</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>https://show.bilibili.com/platform/detail.html?id=93892</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>//i0.hdslb.com/bfs/openplatform/202410/j6UKAzFJ1729216286673.jpeg</t>
         </is>
       </c>
     </row>

</xml_diff>